<commit_message>
feat: implement assessment models and scoring service with factories and migrations
</commit_message>
<xml_diff>
--- a/docs/gantt-minggu-6-12.xlsx
+++ b/docs/gantt-minggu-6-12.xlsx
@@ -123,7 +123,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -211,6 +211,30 @@
         <bgColor rgb="001B365D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000079BF"/>
+        <bgColor rgb="000079BF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C377E0"/>
+        <bgColor rgb="00C377E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
+        <bgColor rgb="00F3F4F6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -282,7 +306,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -524,6 +548,18 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="2" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1437,7 +1473,7 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>UC-13 dashboard petugas data nyata</t>
+          <t>Shell menu 3 peran</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -1445,15 +1481,19 @@
           <t>rencana</t>
         </is>
       </c>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="15" t="n"/>
+      <c r="D19" s="83" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E19" s="83" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="F19" s="15" t="n"/>
       <c r="G19" s="15" t="n"/>
-      <c r="H19" s="14" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="H19" s="84" t="n"/>
       <c r="I19" s="15" t="n"/>
       <c r="J19" s="15" t="n"/>
     </row>
@@ -1953,7 +1993,7 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Shell navigasi statis</t>
+          <t>UC-13 dashboard petugas data nyata</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
@@ -1961,15 +2001,15 @@
           <t>rencana</t>
         </is>
       </c>
-      <c r="D37" s="18" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="D37" s="84" t="n"/>
       <c r="E37" s="15" t="n"/>
       <c r="F37" s="15" t="n"/>
       <c r="G37" s="15" t="n"/>
-      <c r="H37" s="15" t="n"/>
+      <c r="H37" s="85" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I37" s="15" t="n"/>
       <c r="J37" s="15" t="n"/>
     </row>
@@ -1981,7 +2021,7 @@
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>Shell 3 peran + File 11 pivot</t>
+          <t>File 11 pivot program–kategori</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
@@ -3700,7 +3740,7 @@
       </c>
       <c r="B15" s="49" t="inlineStr">
         <is>
-          <t>UC-13 dashboard petugas data nyata</t>
+          <t>Shell menu 3 peran</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
@@ -3711,13 +3751,41 @@
       <c r="D15" s="50" t="n"/>
       <c r="E15" s="50" t="n"/>
       <c r="F15" s="50" t="n"/>
-      <c r="G15" s="50" t="n"/>
-      <c r="H15" s="50" t="n"/>
-      <c r="I15" s="47" t="n"/>
-      <c r="J15" s="47" t="n"/>
-      <c r="K15" s="50" t="n"/>
-      <c r="L15" s="50" t="n"/>
-      <c r="M15" s="50" t="n"/>
+      <c r="G15" s="83" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H15" s="83" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I15" s="83" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J15" s="83" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K15" s="83" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L15" s="83" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="M15" s="83" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="N15" s="50" t="n"/>
       <c r="O15" s="50" t="n"/>
       <c r="P15" s="47" t="n"/>
@@ -3736,41 +3804,13 @@
       <c r="AC15" s="50" t="n"/>
       <c r="AD15" s="47" t="n"/>
       <c r="AE15" s="47" t="n"/>
-      <c r="AF15" s="46" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="AG15" s="46" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="AH15" s="46" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="AI15" s="46" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="AJ15" s="46" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="AK15" s="46" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="AL15" s="46" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="AF15" s="84" t="n"/>
+      <c r="AG15" s="84" t="n"/>
+      <c r="AH15" s="84" t="n"/>
+      <c r="AI15" s="84" t="n"/>
+      <c r="AJ15" s="84" t="n"/>
+      <c r="AK15" s="86" t="n"/>
+      <c r="AL15" s="86" t="n"/>
       <c r="AM15" s="50" t="n"/>
       <c r="AN15" s="50" t="n"/>
       <c r="AO15" s="50" t="n"/>
@@ -5364,7 +5404,7 @@
       </c>
       <c r="B33" s="49" t="inlineStr">
         <is>
-          <t>Shell navigasi statis</t>
+          <t>UC-13 dashboard petugas data nyata</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
@@ -5375,26 +5415,10 @@
       <c r="D33" s="50" t="n"/>
       <c r="E33" s="50" t="n"/>
       <c r="F33" s="50" t="n"/>
-      <c r="G33" s="53" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H33" s="53" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="I33" s="53" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J33" s="53" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G33" s="84" t="n"/>
+      <c r="H33" s="84" t="n"/>
+      <c r="I33" s="86" t="n"/>
+      <c r="J33" s="86" t="n"/>
       <c r="K33" s="50" t="n"/>
       <c r="L33" s="50" t="n"/>
       <c r="M33" s="50" t="n"/>
@@ -5416,13 +5440,41 @@
       <c r="AC33" s="50" t="n"/>
       <c r="AD33" s="47" t="n"/>
       <c r="AE33" s="47" t="n"/>
-      <c r="AF33" s="50" t="n"/>
-      <c r="AG33" s="50" t="n"/>
-      <c r="AH33" s="50" t="n"/>
-      <c r="AI33" s="50" t="n"/>
-      <c r="AJ33" s="50" t="n"/>
-      <c r="AK33" s="47" t="n"/>
-      <c r="AL33" s="47" t="n"/>
+      <c r="AF33" s="85" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="AG33" s="85" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="AH33" s="85" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="AI33" s="85" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="AJ33" s="85" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="AK33" s="85" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="AL33" s="85" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="AM33" s="50" t="n"/>
       <c r="AN33" s="50" t="n"/>
       <c r="AO33" s="50" t="n"/>
@@ -5446,7 +5498,7 @@
       </c>
       <c r="B34" s="44" t="inlineStr">
         <is>
-          <t>Shell 3 peran + File 11 pivot</t>
+          <t>File 11 pivot program–kategori</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -6291,7 +6343,7 @@
       </c>
       <c r="E8" s="56" t="inlineStr">
         <is>
-          <t>File 1 users + File 4 social_accounts</t>
+          <t>File 1 users + File 4 social_accounts · Shell navigasi</t>
         </is>
       </c>
       <c r="F8" s="56" t="n"/>
@@ -6300,11 +6352,7 @@
           <t>File 2 kategori + seeder 5 kategori</t>
         </is>
       </c>
-      <c r="H8" s="56" t="inlineStr">
-        <is>
-          <t>Shell navigasi statis</t>
-        </is>
-      </c>
+      <c r="H8" s="56" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="79" t="n">
@@ -6326,7 +6374,7 @@
       </c>
       <c r="E9" s="56" t="inlineStr">
         <is>
-          <t>File 1 users + File 4 social_accounts</t>
+          <t>File 1 users + File 4 social_accounts · Shell navigasi</t>
         </is>
       </c>
       <c r="F9" s="56" t="n"/>
@@ -6335,11 +6383,7 @@
           <t>File 2 kategori + seeder 5 kategori</t>
         </is>
       </c>
-      <c r="H9" s="56" t="inlineStr">
-        <is>
-          <t>Shell navigasi statis</t>
-        </is>
-      </c>
+      <c r="H9" s="56" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="80" t="n">
@@ -6361,7 +6405,7 @@
       </c>
       <c r="E10" s="60" t="inlineStr">
         <is>
-          <t>File 1 users + File 4 social_accounts</t>
+          <t>File 1 users + File 4 social_accounts · Shell navigasi</t>
         </is>
       </c>
       <c r="F10" s="60" t="inlineStr">
@@ -6374,11 +6418,7 @@
           <t>File 2 kategori + seeder 5 kategori</t>
         </is>
       </c>
-      <c r="H10" s="60" t="inlineStr">
-        <is>
-          <t>Shell navigasi statis</t>
-        </is>
-      </c>
+      <c r="H10" s="60" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="80" t="n">
@@ -6400,7 +6440,7 @@
       </c>
       <c r="E11" s="60" t="inlineStr">
         <is>
-          <t>File 1 users + File 4 social_accounts</t>
+          <t>File 1 users + File 4 social_accounts · Shell navigasi</t>
         </is>
       </c>
       <c r="F11" s="60" t="inlineStr">
@@ -6413,11 +6453,7 @@
           <t>File 2 kategori + seeder 5 kategori</t>
         </is>
       </c>
-      <c r="H11" s="60" t="inlineStr">
-        <is>
-          <t>Shell navigasi statis</t>
-        </is>
-      </c>
+      <c r="H11" s="60" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="79" t="n">
@@ -6439,7 +6475,7 @@
       </c>
       <c r="E12" s="56" t="inlineStr">
         <is>
-          <t>UC-01 login + middleware 3 peran</t>
+          <t>UC-01 login + middleware 3 peran · Shell menu 3 peran</t>
         </is>
       </c>
       <c r="F12" s="56" t="inlineStr">
@@ -6454,7 +6490,7 @@
       </c>
       <c r="H12" s="56" t="inlineStr">
         <is>
-          <t>Shell 3 peran + File 11 pivot</t>
+          <t>File 11 pivot program–kategori</t>
         </is>
       </c>
     </row>
@@ -6478,7 +6514,7 @@
       </c>
       <c r="E13" s="56" t="inlineStr">
         <is>
-          <t>UC-01 login + middleware 3 peran</t>
+          <t>UC-01 login + middleware 3 peran · Shell menu 3 peran</t>
         </is>
       </c>
       <c r="F13" s="56" t="inlineStr">
@@ -6493,7 +6529,7 @@
       </c>
       <c r="H13" s="56" t="inlineStr">
         <is>
-          <t>Shell 3 peran + File 11 pivot</t>
+          <t>File 11 pivot program–kategori</t>
         </is>
       </c>
     </row>
@@ -6517,7 +6553,7 @@
       </c>
       <c r="E14" s="56" t="inlineStr">
         <is>
-          <t>UC-01 login + middleware 3 peran</t>
+          <t>UC-01 login + middleware 3 peran · Shell menu 3 peran</t>
         </is>
       </c>
       <c r="F14" s="56" t="inlineStr">
@@ -6532,7 +6568,7 @@
       </c>
       <c r="H14" s="56" t="inlineStr">
         <is>
-          <t>Shell 3 peran + File 11 pivot</t>
+          <t>File 11 pivot program–kategori</t>
         </is>
       </c>
     </row>
@@ -7256,11 +7292,7 @@
         <f>TRIM(IF(INT(A33)=TODAY(),"hari ini ","")&amp;"")</f>
         <v/>
       </c>
-      <c r="E33" s="56" t="inlineStr">
-        <is>
-          <t>UC-13 dashboard petugas data nyata</t>
-        </is>
-      </c>
+      <c r="E33" s="56" t="n"/>
       <c r="F33" s="56" t="inlineStr">
         <is>
           <t>UC-09b rekomendasi sendiri + dashboard UMKM</t>
@@ -7273,7 +7305,7 @@
       </c>
       <c r="H33" s="56" t="inlineStr">
         <is>
-          <t>UC-10 ajukan + UC-11 setujui/tolak</t>
+          <t>UC-10 ajukan + UC-11 setujui/tolak · UC-13 dashboard petugas data nyata</t>
         </is>
       </c>
     </row>
@@ -7295,11 +7327,7 @@
         <f>TRIM(IF(INT(A34)=TODAY(),"hari ini ","")&amp;"Laporan Selasa — Dashboard data nyata. Ajukan / setujui-tolak")</f>
         <v/>
       </c>
-      <c r="E34" s="56" t="inlineStr">
-        <is>
-          <t>UC-13 dashboard petugas data nyata</t>
-        </is>
-      </c>
+      <c r="E34" s="56" t="n"/>
       <c r="F34" s="56" t="inlineStr">
         <is>
           <t>UC-09b rekomendasi sendiri + dashboard UMKM</t>
@@ -7312,7 +7340,7 @@
       </c>
       <c r="H34" s="56" t="inlineStr">
         <is>
-          <t>UC-10 ajukan + UC-11 setujui/tolak</t>
+          <t>UC-10 ajukan + UC-11 setujui/tolak · UC-13 dashboard petugas data nyata</t>
         </is>
       </c>
     </row>
@@ -7334,11 +7362,7 @@
         <f>TRIM(IF(INT(A35)=TODAY(),"hari ini ","")&amp;"")</f>
         <v/>
       </c>
-      <c r="E35" s="56" t="inlineStr">
-        <is>
-          <t>UC-13 dashboard petugas data nyata</t>
-        </is>
-      </c>
+      <c r="E35" s="56" t="n"/>
       <c r="F35" s="56" t="inlineStr">
         <is>
           <t>UC-09b rekomendasi sendiri + dashboard UMKM</t>
@@ -7351,7 +7375,7 @@
       </c>
       <c r="H35" s="56" t="inlineStr">
         <is>
-          <t>UC-10 ajukan + UC-11 setujui/tolak</t>
+          <t>UC-10 ajukan + UC-11 setujui/tolak · UC-13 dashboard petugas data nyata</t>
         </is>
       </c>
     </row>
@@ -7373,11 +7397,7 @@
         <f>TRIM(IF(INT(A36)=TODAY(),"hari ini ","")&amp;"")</f>
         <v/>
       </c>
-      <c r="E36" s="56" t="inlineStr">
-        <is>
-          <t>UC-13 dashboard petugas data nyata</t>
-        </is>
-      </c>
+      <c r="E36" s="56" t="n"/>
       <c r="F36" s="56" t="inlineStr">
         <is>
           <t>UC-09b rekomendasi sendiri + dashboard UMKM</t>
@@ -7390,7 +7410,7 @@
       </c>
       <c r="H36" s="56" t="inlineStr">
         <is>
-          <t>UC-10 ajukan + UC-11 setujui/tolak</t>
+          <t>UC-10 ajukan + UC-11 setujui/tolak · UC-13 dashboard petugas data nyata</t>
         </is>
       </c>
     </row>
@@ -7412,11 +7432,7 @@
         <f>TRIM(IF(INT(A37)=TODAY(),"hari ini ","")&amp;"")</f>
         <v/>
       </c>
-      <c r="E37" s="56" t="inlineStr">
-        <is>
-          <t>UC-13 dashboard petugas data nyata</t>
-        </is>
-      </c>
+      <c r="E37" s="56" t="n"/>
       <c r="F37" s="56" t="inlineStr">
         <is>
           <t>UC-09b rekomendasi sendiri + dashboard UMKM</t>
@@ -7429,7 +7445,7 @@
       </c>
       <c r="H37" s="56" t="inlineStr">
         <is>
-          <t>UC-10 ajukan + UC-11 setujui/tolak</t>
+          <t>UC-10 ajukan + UC-11 setujui/tolak · UC-13 dashboard petugas data nyata</t>
         </is>
       </c>
     </row>
@@ -7451,11 +7467,7 @@
         <f>TRIM(IF(INT(A38)=TODAY(),"hari ini ","")&amp;"")</f>
         <v/>
       </c>
-      <c r="E38" s="60" t="inlineStr">
-        <is>
-          <t>UC-13 dashboard petugas data nyata</t>
-        </is>
-      </c>
+      <c r="E38" s="60" t="n"/>
       <c r="F38" s="60" t="inlineStr">
         <is>
           <t>UC-09b rekomendasi sendiri + dashboard UMKM</t>
@@ -7468,7 +7480,7 @@
       </c>
       <c r="H38" s="60" t="inlineStr">
         <is>
-          <t>UC-10 ajukan + UC-11 setujui/tolak</t>
+          <t>UC-10 ajukan + UC-11 setujui/tolak · UC-13 dashboard petugas data nyata</t>
         </is>
       </c>
     </row>
@@ -7490,11 +7502,7 @@
         <f>TRIM(IF(INT(A39)=TODAY(),"hari ini ","")&amp;"")</f>
         <v/>
       </c>
-      <c r="E39" s="60" t="inlineStr">
-        <is>
-          <t>UC-13 dashboard petugas data nyata</t>
-        </is>
-      </c>
+      <c r="E39" s="60" t="n"/>
       <c r="F39" s="60" t="inlineStr">
         <is>
           <t>UC-09b rekomendasi sendiri + dashboard UMKM</t>
@@ -7507,7 +7515,7 @@
       </c>
       <c r="H39" s="60" t="inlineStr">
         <is>
-          <t>UC-10 ajukan + UC-11 setujui/tolak</t>
+          <t>UC-10 ajukan + UC-11 setujui/tolak · UC-13 dashboard petugas data nyata</t>
         </is>
       </c>
     </row>
@@ -8134,7 +8142,7 @@
       </c>
       <c r="B4" s="65" t="inlineStr">
         <is>
-          <t>File 1, File 4, login, middleware</t>
+          <t>File 1, File 4, login, middleware, shell menu</t>
         </is>
       </c>
       <c r="C4" s="65" t="inlineStr">
@@ -8144,7 +8152,7 @@
       </c>
       <c r="D4" s="65" t="inlineStr">
         <is>
-          <t>Skor, generate rekomendasi, dashboard petugas nyata</t>
+          <t>Skor, generate rekomendasi</t>
         </is>
       </c>
       <c r="E4" s="65" t="inlineStr">
@@ -8215,7 +8223,7 @@
       </c>
       <c r="B7" s="65" t="inlineStr">
         <is>
-          <t>Shell, File 11, File 12</t>
+          <t>File 11, File 12</t>
         </is>
       </c>
       <c r="C7" s="65" t="inlineStr">
@@ -8225,7 +8233,7 @@
       </c>
       <c r="D7" s="65" t="inlineStr">
         <is>
-          <t>Ajukan, setujui/tolak, File 16</t>
+          <t>UC-13 dashboard petugas, ajukan, setujui/tolak, File 16</t>
         </is>
       </c>
       <c r="E7" s="65" t="inlineStr">

</xml_diff>